<commit_message>
feat: add input/parameter/constant classification in fusion rules
- _compute_fused_io now classifies external inputs as input/parameter/constant
  using module's forward() signature and named_parameters()
- FusionSpec adds parameter_map and constant_map fields
- FusionRule adds parameter_map and constant_map fields
- ModuleTracker adds path_to_module mapping for module inspection
- RMSNorm input_map now correctly shows 1 input (hidden_states) instead of 4
- Add FXTracer (make_fx + decomposition) and FXGraphAdapter (experimental)
- Legacy fusion is primary path, FX tracing is experimental
- Fix _classify_input: only mark Scalar op args > 0 as constant
</commit_message>
<xml_diff>
--- a/deepseek_v3_2_ops.xlsx
+++ b/deepseek_v3_2_ops.xlsx
@@ -962,7 +962,7 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>embedding[0] | embedding[1]</t>
+          <t>embedding[0](param:weight) | embedding[1]</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | add[0] | mul[0] | mul[1]</t>
+          <t>pow[0] | add[0] | mul[0](param:weight) | mul[1]</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 1536], [1, 128, 1536], [1536], [1, 128, 1536]</t>
+          <t>[1, 128, 1536], [1, 128, 1536], [1, 128, 1], [1536]</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -1170,12 +1170,24 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | mul[0] | mul[1]</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
+          <t>pow[0] | mean[0] | add[0] | mul[0](param:weight)</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>[1, 128, 1536]</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>mul[0]</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -1201,34 +1213,22 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>[128, 1536]</t>
+          <t>[128, 1536], [1536, 24576]</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>torch.float32</t>
+          <t>torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>mm[0]</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>[128, 24576]</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>mm[0]</t>
-        </is>
-      </c>
+          <t>mm[0] | mm[1]</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -1267,9 +1267,21 @@
           <t>transpose[0]</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
-      <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>[1, 128, 128, 192]</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>transpose[0]</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -1308,21 +1320,9 @@
           <t>mm[0] | mm[1]</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>[128, 576]</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>mm[0]</t>
-        </is>
-      </c>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1401,17 +1401,17 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 512], [1, 128, 512], [1, 128, 1], [512]</t>
+          <t>[1, 128, 512], [1, 128, 512], [1, 128, 1], [512], [1, 128, 512]</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | mul[0]</t>
+          <t>pow[0] | mean[0] | add[0] | mul[0](param:weight) | mul[1]</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr"/>
@@ -1442,17 +1442,17 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>[128, 512]</t>
+          <t>[128, 512], [512, 32768]</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>torch.float32</t>
+          <t>torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>mm[0]</t>
+          <t>mm[0] | mm[1]</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1508,9 +1508,21 @@
           <t>transpose[0]</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr"/>
-      <c r="J13" s="4" t="inlineStr"/>
-      <c r="K13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>[1, 128, 128, 256]</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>transpose[0]</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1589,17 +1601,17 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 1536], [1, 128, 1536], [1536]</t>
+          <t>[1, 128, 1536], [1, 128, 1536], [1536], [1, 128, 1536]</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | mul[0]</t>
+          <t>pow[0] | mean[0] | mul[0](param:weight) | mul[1]</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1655,9 +1667,21 @@
           <t>mm[0]</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>[128, 8192]</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>mm[0]</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1746,7 +1770,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>mm[0] | mm[1]</t>
+          <t>mm[0](param:weight) | mm[1]</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1799,7 +1823,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>native_layer_norm[0] | native_layer_norm[1] | native_layer_norm[2]</t>
+          <t>native_layer_norm[0] | native_layer_norm[1](param:weight) | native_layer_norm[2](param:weight)</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
@@ -1895,7 +1919,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>[32], [32], [128, 32], [128, 64]</t>
+          <t>[32], [32], [32], [128, 1]</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1905,22 +1929,22 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>reciprocal[0] | mul[0] | cat[0] | mul[0]</t>
+          <t>div[0] | reciprocal[0] | div[0] | mul[0]</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>[128, 64]</t>
+          <t>[128, 64], [128, 64]</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>torch.float32</t>
+          <t>torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>mul[0]</t>
+          <t>mul[0] | mul[0]</t>
         </is>
       </c>
     </row>
@@ -1948,34 +1972,22 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>[128, 64], [1, 128], [128, 64], [1, 128, 128, 128], [1, 128, 128, 128], [1, 128, 128, 128], [1, 1, 128, 128], [128, 128, 128], [1, 128, 128, 128]</t>
+          <t>[128, 64], [1, 128], [128, 64], [1, 1, 128, 64], [1, 128, 128, 128], [1, 128, 128, 128], [1, 128, 128, 128], [1, 1, 128, 128], [128, 128, 128], [1, 128, 128, 128]</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.int64, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.int64, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>index[0] | index[1] | index[0] | copy_[1] | copy_[1] | add[0] | add[1] | bmm[0] | transpose[0]</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>[1, 128, 64]</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>index[0]</t>
-        </is>
-      </c>
+          <t>index[0] | index[1] | index[0] | mul[0] | copy_[1] | copy_[1] | add[0] | add[1] | bmm[0] | transpose[0]</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr"/>
+      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -2107,17 +2119,17 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [7168], [1, 128, 7168]</t>
+          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [7168]</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[0] | mul[1]</t>
+          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr"/>
@@ -2214,9 +2226,21 @@
           <t>silu[0]</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr"/>
-      <c r="J27" s="4" t="inlineStr"/>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>[1, 128, 18432]</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>silu[0]</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -2255,21 +2279,9 @@
           <t>mm[0] | mm[1]</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>[128, 18432]</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>mm[0]</t>
-        </is>
-      </c>
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -2308,9 +2320,21 @@
           <t>mul[0] | mul[1]</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr"/>
-      <c r="K29" s="4" t="inlineStr"/>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>[1, 128, 18432]</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>mul[0]</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -2442,17 +2466,17 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [1, 128, 1], [7168], [1, 128, 7168]</t>
+          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [7168], [1, 128, 7168]</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[1] | mul[0] | mul[1]</t>
+          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[0](param:weight) | mul[1]</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr"/>
@@ -2536,17 +2560,17 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 1536], [1, 128, 1536], [1, 128, 1], [1, 128, 1], [1536], [1, 128, 1536]</t>
+          <t>[1, 128, 1536], [1, 128, 1536], [1, 128, 1], [1, 128, 1], [1536]</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | mul[1] | mul[0] | mul[1]</t>
+          <t>pow[0] | mean[0] | add[0] | mul[1] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -2602,21 +2626,9 @@
           <t>mm[0] | mm[1]</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>[128, 24576]</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K35" s="4" t="inlineStr">
-        <is>
-          <t>mm[0]</t>
-        </is>
-      </c>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -2708,9 +2720,21 @@
           <t>mm[0] | mm[1]</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr"/>
-      <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>[128, 576]</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>mm[0]</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -2789,17 +2813,17 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 512], [1, 128, 512], [512]</t>
+          <t>[1, 128, 512], [1, 128, 512], [1, 128, 1], [512]</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | mul[0]</t>
+          <t>pow[0] | mean[0] | add[0] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr"/>
@@ -2987,12 +3011,24 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | mul[0] | mul[1]</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="inlineStr"/>
-      <c r="J43" s="4" t="inlineStr"/>
-      <c r="K43" s="4" t="inlineStr"/>
+          <t>pow[0] | mean[0] | mul[0](param:weight) | mul[1]</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>[1, 128, 1536]</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>mul[0]</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -3134,7 +3170,7 @@
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>mm[0] | mm[1]</t>
+          <t>mm[0](param:weight) | mm[1]</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -3187,7 +3223,7 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>native_layer_norm[0] | native_layer_norm[1] | native_layer_norm[2]</t>
+          <t>native_layer_norm[0] | native_layer_norm[1](param:weight) | native_layer_norm[2](param:weight)</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
@@ -3336,34 +3372,22 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>[128, 64], [1, 128], [128, 64], [1, 1, 128, 64], [1, 128, 128, 128], [1, 128, 128, 64], [1, 128, 128, 128], [1, 128, 128, 128], [1, 1, 128, 128], [128, 128, 128]</t>
+          <t>[128, 64], [1, 128], [128, 64], [1, 1, 128, 64], [1, 128, 128, 128], [1, 128, 128, 128], [1, 1, 128, 128], [128, 128, 128], [1, 128, 128, 128]</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.int64, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.int64, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>index[0] | index[1] | index[0] | mul[0] | copy_[1] | copy_[1] | copy_[1] | add[0] | add[1] | bmm[0]</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="inlineStr">
-        <is>
-          <t>[1, 128, 128, 192]</t>
-        </is>
-      </c>
-      <c r="J50" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K50" s="4" t="inlineStr">
-        <is>
-          <t>new_empty[0]</t>
-        </is>
-      </c>
+          <t>index[0] | index[1] | index[0] | mul[0] | copy_[1] | copy_[1] | add[1] | bmm[0] | transpose[0]</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr"/>
+      <c r="J50" s="4" t="inlineStr"/>
+      <c r="K50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -3389,34 +3413,22 @@
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>[128, 16384]</t>
+          <t>[128, 16384], [16384, 7168]</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>torch.float32</t>
+          <t>torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>mm[0]</t>
-        </is>
-      </c>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>[128, 7168]</t>
-        </is>
-      </c>
-      <c r="J51" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K51" s="4" t="inlineStr">
-        <is>
-          <t>mm[0]</t>
-        </is>
-      </c>
+          <t>mm[0] | mm[1]</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="inlineStr"/>
+      <c r="K51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -3495,17 +3507,17 @@
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [7168], [1, 128, 7168]</t>
+          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [7168]</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[0] | mul[1]</t>
+          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr"/>
@@ -3830,17 +3842,17 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [1, 128, 1], [7168], [1, 128, 7168]</t>
+          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [1, 128, 1], [7168]</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[1] | mul[0] | mul[1]</t>
+          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[1] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr"/>
@@ -3924,7 +3936,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 1536], [1, 128, 1536], [1, 128, 1], [1, 128, 1], [1536], [1, 128, 1536]</t>
+          <t>[1, 128, 1536], [1, 128, 1536], [1, 128, 1], [1, 128, 1], [1, 128, 1], [1536]</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -3934,7 +3946,7 @@
       </c>
       <c r="H62" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | mul[1] | mul[0] | mul[1]</t>
+          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[1] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I62" s="4" t="inlineStr">
@@ -4187,7 +4199,7 @@
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | mul[0]</t>
+          <t>pow[0] | mean[0] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr"/>
@@ -4375,24 +4387,12 @@
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | mul[0] | mul[1]</t>
-        </is>
-      </c>
-      <c r="I71" s="4" t="inlineStr">
-        <is>
-          <t>[1, 128, 1536]</t>
-        </is>
-      </c>
-      <c r="J71" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K71" s="4" t="inlineStr">
-        <is>
-          <t>mul[0]</t>
-        </is>
-      </c>
+          <t>pow[0] | mean[0] | mul[0](param:weight) | mul[1]</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="inlineStr"/>
+      <c r="J71" s="4" t="inlineStr"/>
+      <c r="K71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -4534,7 +4534,7 @@
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>mm[0] | mm[1]</t>
+          <t>mm[0](param:weight) | mm[1]</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
@@ -4587,22 +4587,22 @@
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>native_layer_norm[0] | native_layer_norm[1] | native_layer_norm[2]</t>
+          <t>native_layer_norm[0] | native_layer_norm[1](param:weight) | native_layer_norm[2](param:weight)</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 1], [1, 128, 128]</t>
+          <t>[1, 128, 1]</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32</t>
+          <t>torch.float32</t>
         </is>
       </c>
       <c r="K75" s="4" t="inlineStr">
         <is>
-          <t>native_layer_norm[2] | native_layer_norm[0]</t>
+          <t>native_layer_norm[1]</t>
         </is>
       </c>
     </row>
@@ -4630,17 +4630,17 @@
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>[1, 64, 128, 64], [1, 64, 128, 128], [1, 1, 128, 128]</t>
+          <t>[1, 64, 128, 128], [1, 1, 128, 128]</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
-          <t>transpose[0] | add[0] | add[1]</t>
+          <t>add[0] | add[1]</t>
         </is>
       </c>
       <c r="I76" s="4" t="inlineStr">
@@ -4683,32 +4683,32 @@
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>[32], [32], [32], [128, 64], [128, 64]</t>
+          <t>[32], [32], [32], [128, 1]</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mul[0] | mul[0] | cos[0] | mul[0]</t>
+          <t>div[0] | reciprocal[0] | div[0] | mul[0]</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>[128, 64]</t>
+          <t>[128, 64], [128, 64]</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
-          <t>torch.float32</t>
+          <t>torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="K77" s="4" t="inlineStr">
         <is>
-          <t>mul[0]</t>
+          <t>mul[0] | mul[0]</t>
         </is>
       </c>
     </row>
@@ -4736,22 +4736,34 @@
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>[128, 64], [1, 128], [128, 64], [1, 128, 128, 128], [1, 128, 128, 128], [1, 128, 128, 128], [1, 1, 128, 128], [128, 128, 128]</t>
+          <t>[128, 64], [1, 128], [128, 64], [1, 1, 128, 64], [1, 1, 128, 64], [1, 128, 128, 128], [1, 128, 128, 64], [1, 128, 128, 128], [1, 128, 128, 128], [1, 1, 128, 128]</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.int64, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.int64, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
-          <t>index[0] | index[1] | index[0] | copy_[1] | copy_[1] | add[0] | add[1] | bmm[0]</t>
-        </is>
-      </c>
-      <c r="I78" s="4" t="inlineStr"/>
-      <c r="J78" s="4" t="inlineStr"/>
-      <c r="K78" s="4" t="inlineStr"/>
+          <t>index[0] | index[1] | index[0] | mul[0] | new_empty[0] | copy_[1] | copy_[1] | copy_[1] | add[0] | add[1]</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>[1, 128, 128, 192]</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K78" s="4" t="inlineStr">
+        <is>
+          <t>new_empty[0]</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
@@ -4883,17 +4895,17 @@
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [7168], [1, 128, 7168]</t>
+          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [7168], [1, 128, 7168]</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | mul[0] | mul[1]</t>
+          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[0](param:weight) | mul[1]</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr"/>
@@ -4937,9 +4949,21 @@
           <t>mm[0] | mm[1]</t>
         </is>
       </c>
-      <c r="I82" s="4" t="inlineStr"/>
-      <c r="J82" s="4" t="inlineStr"/>
-      <c r="K82" s="4" t="inlineStr"/>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>[128, 18432]</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K82" s="4" t="inlineStr">
+        <is>
+          <t>mm[0]</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n">
@@ -5031,9 +5055,21 @@
           <t>mm[0] | mm[1]</t>
         </is>
       </c>
-      <c r="I84" s="4" t="inlineStr"/>
-      <c r="J84" s="4" t="inlineStr"/>
-      <c r="K84" s="4" t="inlineStr"/>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>[128, 18432]</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="inlineStr">
+        <is>
+          <t>mm[0]</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
@@ -5072,9 +5108,21 @@
           <t>mul[0] | mul[1]</t>
         </is>
       </c>
-      <c r="I85" s="4" t="inlineStr"/>
-      <c r="J85" s="4" t="inlineStr"/>
-      <c r="K85" s="4" t="inlineStr"/>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>[1, 128, 18432]</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K85" s="4" t="inlineStr">
+        <is>
+          <t>mul[0]</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n">
@@ -5206,17 +5254,17 @@
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [1, 128, 1], [7168], [1, 128, 7168]</t>
+          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [1, 128, 1], [7168]</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[1] | mul[0] | mul[1]</t>
+          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[1] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I88" s="4" t="inlineStr"/>
@@ -5300,17 +5348,17 @@
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 1536], [1, 128, 1536], [1, 128, 1], [1536], [1, 128, 1536]</t>
+          <t>[1, 128, 1536], [1, 128, 1536], [1, 128, 1], [1536]</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | mul[1] | mul[0] | mul[1]</t>
+          <t>pow[0] | mean[0] | add[0] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I90" s="4" t="inlineStr"/>
@@ -5354,21 +5402,9 @@
           <t>mm[0] | mm[1]</t>
         </is>
       </c>
-      <c r="I91" s="4" t="inlineStr">
-        <is>
-          <t>[128, 24576]</t>
-        </is>
-      </c>
-      <c r="J91" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K91" s="4" t="inlineStr">
-        <is>
-          <t>mm[0]</t>
-        </is>
-      </c>
+      <c r="I91" s="4" t="inlineStr"/>
+      <c r="J91" s="4" t="inlineStr"/>
+      <c r="K91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n">
@@ -5448,21 +5484,9 @@
           <t>mm[0] | mm[1]</t>
         </is>
       </c>
-      <c r="I93" s="4" t="inlineStr">
-        <is>
-          <t>[128, 576]</t>
-        </is>
-      </c>
-      <c r="J93" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K93" s="4" t="inlineStr">
-        <is>
-          <t>mm[0]</t>
-        </is>
-      </c>
+      <c r="I93" s="4" t="inlineStr"/>
+      <c r="J93" s="4" t="inlineStr"/>
+      <c r="K93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n">
@@ -5501,21 +5525,9 @@
           <t>transpose[0]</t>
         </is>
       </c>
-      <c r="I94" s="4" t="inlineStr">
-        <is>
-          <t>[1, 1, 128, 64]</t>
-        </is>
-      </c>
-      <c r="J94" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K94" s="4" t="inlineStr">
-        <is>
-          <t>transpose[0]</t>
-        </is>
-      </c>
+      <c r="I94" s="4" t="inlineStr"/>
+      <c r="J94" s="4" t="inlineStr"/>
+      <c r="K94" s="4" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
@@ -5551,7 +5563,7 @@
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | mul[0]</t>
+          <t>pow[0] | mean[0] | add[0] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr"/>
@@ -5582,17 +5594,17 @@
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>[128, 512]</t>
+          <t>[128, 512], [512, 32768]</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>torch.float32</t>
+          <t>torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H96" s="4" t="inlineStr">
         <is>
-          <t>mm[0]</t>
+          <t>mm[0] | mm[1]</t>
         </is>
       </c>
       <c r="I96" s="4" t="inlineStr">
@@ -5648,9 +5660,21 @@
           <t>transpose[0]</t>
         </is>
       </c>
-      <c r="I97" s="4" t="inlineStr"/>
-      <c r="J97" s="4" t="inlineStr"/>
-      <c r="K97" s="4" t="inlineStr"/>
+      <c r="I97" s="4" t="inlineStr">
+        <is>
+          <t>[1, 128, 128, 256]</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K97" s="4" t="inlineStr">
+        <is>
+          <t>transpose[0]</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n">
@@ -5739,12 +5763,24 @@
       </c>
       <c r="H99" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | mul[0] | mul[1]</t>
-        </is>
-      </c>
-      <c r="I99" s="4" t="inlineStr"/>
-      <c r="J99" s="4" t="inlineStr"/>
-      <c r="K99" s="4" t="inlineStr"/>
+          <t>pow[0] | mean[0] | mul[0](param:weight) | mul[1]</t>
+        </is>
+      </c>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>[1, 128, 1536]</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K99" s="4" t="inlineStr">
+        <is>
+          <t>mul[0]</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n">
@@ -5886,7 +5922,7 @@
       </c>
       <c r="H102" s="4" t="inlineStr">
         <is>
-          <t>mm[0] | mm[1]</t>
+          <t>mm[0](param:weight) | mm[1]</t>
         </is>
       </c>
       <c r="I102" s="4" t="inlineStr">
@@ -5939,7 +5975,7 @@
       </c>
       <c r="H103" s="4" t="inlineStr">
         <is>
-          <t>native_layer_norm[0] | native_layer_norm[1] | native_layer_norm[2]</t>
+          <t>native_layer_norm[0] | native_layer_norm[1](param:weight) | native_layer_norm[2](param:weight)</t>
         </is>
       </c>
       <c r="I103" s="4" t="inlineStr">
@@ -6088,34 +6124,22 @@
       </c>
       <c r="F106" s="4" t="inlineStr">
         <is>
-          <t>[128, 64], [1, 128], [128, 64], [1, 1, 128, 64], [1, 128, 128, 128], [1, 128, 128, 64], [1, 128, 128, 128], [1, 1, 128, 128], [128, 128, 128], [128, 128, 128]</t>
+          <t>[128, 64], [1, 128], [128, 64], [1, 1, 128, 64], [1, 128, 128, 128], [1, 128, 128, 64], [1, 1, 128, 128], [128, 128, 128], [128, 128, 128]</t>
         </is>
       </c>
       <c r="G106" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.int64, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.int64, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H106" s="4" t="inlineStr">
         <is>
-          <t>index[0] | index[1] | index[0] | mul[0] | copy_[1] | copy_[1] | copy_[1] | add[1] | bmm[0] | bmm[1]</t>
-        </is>
-      </c>
-      <c r="I106" s="4" t="inlineStr">
-        <is>
-          <t>[1, 128, 128, 192], [128, 128, 128]</t>
-        </is>
-      </c>
-      <c r="J106" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32, torch.float32</t>
-        </is>
-      </c>
-      <c r="K106" s="4" t="inlineStr">
-        <is>
-          <t>new_empty[0] | bmm[0]</t>
-        </is>
-      </c>
+          <t>index[0] | index[1] | index[0] | mul[0] | copy_[1] | copy_[1] | add[1] | bmm[0] | bmm[1]</t>
+        </is>
+      </c>
+      <c r="I106" s="4" t="inlineStr"/>
+      <c r="J106" s="4" t="inlineStr"/>
+      <c r="K106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n">
@@ -6141,34 +6165,22 @@
       </c>
       <c r="F107" s="4" t="inlineStr">
         <is>
-          <t>[128, 16384], [16384, 7168]</t>
+          <t>[128, 16384]</t>
         </is>
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32</t>
+          <t>torch.float32</t>
         </is>
       </c>
       <c r="H107" s="4" t="inlineStr">
         <is>
-          <t>mm[0] | mm[1]</t>
-        </is>
-      </c>
-      <c r="I107" s="4" t="inlineStr">
-        <is>
-          <t>[128, 7168]</t>
-        </is>
-      </c>
-      <c r="J107" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K107" s="4" t="inlineStr">
-        <is>
           <t>mm[0]</t>
         </is>
       </c>
+      <c r="I107" s="4" t="inlineStr"/>
+      <c r="J107" s="4" t="inlineStr"/>
+      <c r="K107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n">
@@ -6247,17 +6259,17 @@
       </c>
       <c r="F109" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [1, 128, 1], [7168]</t>
+          <t>[1, 128, 7168], [1, 128, 7168], [1, 128, 1], [7168]</t>
         </is>
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mean[0] | add[0] | rsqrt[0] | mul[0]</t>
+          <t>pow[0] | mean[0] | rsqrt[0] | mul[0](param:weight)</t>
         </is>
       </c>
       <c r="I109" s="4" t="inlineStr"/>
@@ -6288,32 +6300,32 @@
       </c>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>[128, 7168], [128, 256], [128, 256], [128, 1]</t>
+          <t>[128, 7168], [7168, 256], [128, 256], [1, 256], [128, 8], [128, 8], [128, 1]</t>
         </is>
       </c>
       <c r="G110" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.bool, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.int64, torch.float32</t>
         </is>
       </c>
       <c r="H110" s="4" t="inlineStr">
         <is>
-          <t>mm[0] | sigmoid[0] | masked_fill[1] | add[0]</t>
+          <t>mm[0] | mm[1] | sigmoid[0] | add[1] | topk[0] | gather[1] | add[0]</t>
         </is>
       </c>
       <c r="I110" s="4" t="inlineStr">
         <is>
-          <t>[128, 256], [128, 8]</t>
+          <t>[128, 8]</t>
         </is>
       </c>
       <c r="J110" s="4" t="inlineStr">
         <is>
-          <t>torch.bool, torch.float32</t>
+          <t>torch.float32</t>
         </is>
       </c>
       <c r="K110" s="4" t="inlineStr">
         <is>
-          <t>_to_copy[0] | mul[0]</t>
+          <t>mul[0]</t>
         </is>
       </c>
     </row>
@@ -6341,17 +6353,17 @@
       </c>
       <c r="F111" s="4" t="inlineStr">
         <is>
-          <t>[128, 7168]</t>
+          <t>[128, 7168], [7168, 2048]</t>
         </is>
       </c>
       <c r="G111" s="4" t="inlineStr">
         <is>
-          <t>torch.float32</t>
+          <t>torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H111" s="4" t="inlineStr">
         <is>
-          <t>mm[0]</t>
+          <t>mm[0] | mm[1]</t>
         </is>
       </c>
       <c r="I111" s="4" t="inlineStr">
@@ -6460,9 +6472,21 @@
           <t>mm[0] | mm[1]</t>
         </is>
       </c>
-      <c r="I113" s="4" t="inlineStr"/>
-      <c r="J113" s="4" t="inlineStr"/>
-      <c r="K113" s="4" t="inlineStr"/>
+      <c r="I113" s="4" t="inlineStr">
+        <is>
+          <t>[128, 2048]</t>
+        </is>
+      </c>
+      <c r="J113" s="4" t="inlineStr">
+        <is>
+          <t>torch.float32</t>
+        </is>
+      </c>
+      <c r="K113" s="4" t="inlineStr">
+        <is>
+          <t>mm[0]</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="n">
@@ -6501,21 +6525,9 @@
           <t>mul[0] | mul[1]</t>
         </is>
       </c>
-      <c r="I114" s="4" t="inlineStr">
-        <is>
-          <t>[128, 2048]</t>
-        </is>
-      </c>
-      <c r="J114" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K114" s="4" t="inlineStr">
-        <is>
-          <t>mul[0]</t>
-        </is>
-      </c>
+      <c r="I114" s="4" t="inlineStr"/>
+      <c r="J114" s="4" t="inlineStr"/>
+      <c r="K114" s="4" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="n">
@@ -6554,21 +6566,9 @@
           <t>mm[0] | mm[1]</t>
         </is>
       </c>
-      <c r="I115" s="4" t="inlineStr">
-        <is>
-          <t>[128, 7168]</t>
-        </is>
-      </c>
-      <c r="J115" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="K115" s="4" t="inlineStr">
-        <is>
-          <t>mm[0]</t>
-        </is>
-      </c>
+      <c r="I115" s="4" t="inlineStr"/>
+      <c r="J115" s="4" t="inlineStr"/>
+      <c r="K115" s="4" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="3" t="n">
@@ -6978,17 +6978,17 @@
       <c r="E124" s="4" t="inlineStr"/>
       <c r="F124" s="4" t="inlineStr">
         <is>
-          <t>[1, 128, 7168], [1, 128, 1], [7168]</t>
+          <t>[1, 128, 7168], [1, 128, 1], [1, 128, 1], [7168], [1, 128, 7168]</t>
         </is>
       </c>
       <c r="G124" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="H124" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | mul[1] | mul[0]</t>
+          <t>pow[0] | add[0] | mul[1] | mul[0](param:weight) | mul[1]</t>
         </is>
       </c>
       <c r="I124" s="4" t="inlineStr">
@@ -28732,7 +28732,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>pow[0] | add[0] | mul[0] | mul[1]</t>
+          <t>pow[0] | add[0] | mul[0](param:weight) | mul[1]</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -28838,7 +28838,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>[32], [32], [128, 32], [128, 64]</t>
+          <t>[32], [32], [32], [128, 1]</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -28848,22 +28848,22 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>reciprocal[0] | mul[0] | cat[0] | mul[0]</t>
+          <t>div[0] | reciprocal[0] | div[0] | mul[0]</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>[128, 64]</t>
+          <t>[128, 64], [128, 64]</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>torch.float32</t>
+          <t>torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>mul[0]</t>
+          <t>mul[0] | mul[0]</t>
         </is>
       </c>
     </row>
@@ -28896,34 +28896,22 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>[128, 64], [1, 128], [128, 64], [1, 128, 128, 128], [1, 128, 128, 128], [1, 128, 128, 128], [1, 1, 128, 128], [128, 128, 128], [1, 128, 128, 128]</t>
+          <t>[128, 64], [1, 128], [128, 64], [1, 1, 128, 64], [1, 128, 128, 128], [1, 128, 128, 128], [1, 128, 128, 128], [1, 1, 128, 128], [128, 128, 128], [1, 128, 128, 128]</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.int64, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
+          <t>torch.float32, torch.int64, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.float32</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>index[0] | index[1] | index[0] | copy_[1] | copy_[1] | add[0] | add[1] | bmm[0] | transpose[0]</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>[1, 128, 64]</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>torch.float32</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>index[0]</t>
-        </is>
-      </c>
+          <t>index[0] | index[1] | index[0] | mul[0] | copy_[1] | copy_[1] | add[0] | add[1] | bmm[0] | transpose[0]</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -29012,32 +29000,32 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>[128, 7168], [128, 256], [128, 256], [128, 1]</t>
+          <t>[128, 7168], [7168, 256], [128, 256], [1, 256], [128, 8], [128, 8], [128, 1]</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>torch.float32, torch.float32, torch.bool, torch.float32</t>
+          <t>torch.float32, torch.float32, torch.float32, torch.float32, torch.float32, torch.int64, torch.float32</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>mm[0] | sigmoid[0] | masked_fill[1] | add[0]</t>
+          <t>mm[0] | mm[1] | sigmoid[0] | add[1] | topk[0] | gather[1] | add[0]</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>[128, 256], [128, 8]</t>
+          <t>[128, 8]</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>torch.bool, torch.float32</t>
+          <t>torch.float32</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>_to_copy[0] | mul[0]</t>
+          <t>mul[0]</t>
         </is>
       </c>
     </row>

</xml_diff>